<commit_message>
Auto commit 05-07-2025  1:01:55.30
</commit_message>
<xml_diff>
--- a/Templates/110 mm Borewell Construction.xlsx
+++ b/Templates/110 mm Borewell Construction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Core i5 GAMING\Desktop\estimate-drafter\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{1E47E775-D7D5-4E1C-AE26-42E6853710BD}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{2E65A5D3-7E33-49F7-95C2-D8ADDD3B0A1E}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>110mm (4.5") Borewell Drilling (Code: GWDDR100)</t>
   </si>
@@ -30,17 +30,27 @@
   <si>
     <t>PVC End cap 140 mm (DG) (Code: GWDMR003)</t>
   </si>
+  <si>
+    <t>Supplying, assembling, lowering and fixing in vertical position in Borewell, PVC 110 mm 6 Kg/cm2 well casing pipe of required dia, conforming to IS : 4985:2000, including required hire and labour charges, fittings &amp; accessories etc. all complete, for all depths, as per direction of Engineer- in- Charge. (Code: GWDDR014)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -85,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -93,13 +103,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -416,7 +429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13167D5F-AA8D-42F0-9D42-F4CD58E1B9A5}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="44.28515625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="68.140625" style="5" customWidth="1"/>
@@ -440,11 +453,19 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B4" s="3">
         <v>1</v>
       </c>
     </row>

</xml_diff>